<commit_message>
Fix PM Excel Press asset matching
</commit_message>
<xml_diff>
--- a/tests/fixtures/pm-report-sanitized.xlsx
+++ b/tests/fixtures/pm-report-sanitized.xlsx
@@ -24,7 +24,7 @@
     <t>Press:</t>
   </si>
   <si>
-    <t>M-100</t>
+    <t>100</t>
   </si>
   <si>
     <t/>
@@ -82,7 +82,7 @@
     <t>Annual safety review</t>
   </si>
   <si>
-    <t>M-200</t>
+    <t>200</t>
   </si>
   <si>
     <t>Sanitized Press B</t>

</xml_diff>